<commit_message>
Add Interflon Impulse Connect (7213) option, 3D visualization & DB entry, remove 6mm from remote selector, fix brochure button
</commit_message>
<xml_diff>
--- a/odoo_koppelingen_import_v2.xlsx
+++ b/odoo_koppelingen_import_v2.xlsx
@@ -3125,7 +3125,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G31"/>
+  <dimension ref="A1:G32"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="15" customWidth="1" min="1" max="1"/>
@@ -4284,6 +4284,43 @@
         </is>
       </c>
     </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>7213</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>Interflon Impulse Connect (Drukversterker 10 bar + Bluetooth)</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>Booster</t>
+        </is>
+      </c>
+      <c r="D32" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="E32" t="inlineStr">
+        <is>
+          <t>G 1/4" F naar G 1/4" M</t>
+        </is>
+      </c>
+      <c r="F32" t="inlineStr">
+        <is>
+          <t>Kunststof / RVS (IP68)</t>
+        </is>
+      </c>
+      <c r="G32" t="inlineStr">
+        <is>
+          <t>Elektromechanische drukversterker tot 10 bar met Bluetooth connectiviteit en geintegreerde terugslagklep, montage direct onder ISPL (art. 7213)</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Integratie Pulsarlube modellen (M2, BT, MSP, PLC, OL500, MSP Oil), multi-point verdeelblokken 2-8 poorten, borstelsets, dupliceren van smeerpunten en aantalvermenigvuldiger
</commit_message>
<xml_diff>
--- a/odoo_koppelingen_import_v2.xlsx
+++ b/odoo_koppelingen_import_v2.xlsx
@@ -9,6 +9,7 @@
   <sheets>
     <sheet name="Koppelingen &amp; Kits" sheetId="1" state="visible" r:id="rId1"/>
     <sheet name="ISPL Smeerunits" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Pulsarlube" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -4324,4 +4325,3496 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:I74"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>Art. Code (Odoo)</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>Categorie</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>Model / Onderdeelnaam</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>Inhoud / Volume</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>Vettype / Smeermiddel</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>Aansluiting 1 (Inlaat / Boven)</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>Aansluiting 2 (Uitlaat / Onder)</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>Materiaal / Eigenschappen</t>
+        </is>
+      </c>
+      <c r="I1" t="inlineStr">
+        <is>
+          <t>Toelichting / Specificatie</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>1422</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>Dispensers (Vet)</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>Pulsarlube M2 (60 ml)</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>60 ml</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>Herbruikbaar elektro-mechanisch</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>G 3/8" M (of adapter 1/8" NPT)</t>
+        </is>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>Kunststof / RVS (IP65)</t>
+        </is>
+      </c>
+      <c r="I2" t="inlineStr">
+        <is>
+          <t>Elektro-mechanische automatische smeerunit 30-60 bar (art. 1422)</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>1423</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Dispensers (Vet)</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>Pulsarlube M2 (125 ml)</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>125 ml</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>Herbruikbaar elektro-mechanisch</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>G 3/8" M (of adapter 1/8" NPT)</t>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>Kunststof / RVS (IP65)</t>
+        </is>
+      </c>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>Elektro-mechanische automatische smeerunit 30-60 bar (art. 1423)</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>1424</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Dispensers (Vet)</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>Pulsarlube M2 (250 ml)</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>250 ml</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>Herbruikbaar elektro-mechanisch</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>G 3/8" M (of adapter 1/8" NPT)</t>
+        </is>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>Kunststof / RVS (IP65)</t>
+        </is>
+      </c>
+      <c r="I4" t="inlineStr">
+        <is>
+          <t>Elektro-mechanische automatische smeerunit 30-60 bar (art. 1424)</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>1425</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Dispensers (Vet)</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>Pulsarlube M2 (500 ml)</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>500 ml</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>Herbruikbaar elektro-mechanisch</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>G 3/8" M (of adapter 1/8" NPT)</t>
+        </is>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>Kunststof / RVS (IP65)</t>
+        </is>
+      </c>
+      <c r="I5" t="inlineStr">
+        <is>
+          <t>Elektro-mechanische automatische smeerunit 30-60 bar (art. 1425)</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>1477</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>Dispensers (Vet)</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>Pulsarlube BT (60 ml)</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>60 ml</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>Bluetooth BLE connectiviteit</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>G 3/8" M (of adapter 1/8" NPT)</t>
+        </is>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>Kunststof / RVS (IP65)</t>
+        </is>
+      </c>
+      <c r="I6" t="inlineStr">
+        <is>
+          <t>Draadloos bewaakte automatische smeerunit via Bluetooth app (art. 1477)</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>1478</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>Dispensers (Vet)</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>Pulsarlube BT (120 ml)</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>120 ml</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>Bluetooth BLE connectiviteit</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>G 3/8" M (of adapter 1/8" NPT)</t>
+        </is>
+      </c>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>Kunststof / RVS (IP65)</t>
+        </is>
+      </c>
+      <c r="I7" t="inlineStr">
+        <is>
+          <t>Draadloos bewaakte automatische smeerunit via Bluetooth app (art. 1478)</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>1479</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>Dispensers (Vet)</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>Pulsarlube BT (240 ml)</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>240 ml</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>Bluetooth BLE connectiviteit</t>
+        </is>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>G 3/8" M (of adapter 1/8" NPT)</t>
+        </is>
+      </c>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>Kunststof / RVS (IP65)</t>
+        </is>
+      </c>
+      <c r="I8" t="inlineStr">
+        <is>
+          <t>Draadloos bewaakte automatische smeerunit via Bluetooth app (art. 1479)</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>1448</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>Dispensers (Vet)</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>Pulsarlube MSP AC (60 ml)</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>60 ml</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>Extern gevoed AC</t>
+        </is>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>G 3/8" M (of adapter 1/8" NPT)</t>
+        </is>
+      </c>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>Kunststof / RVS (IP65)</t>
+        </is>
+      </c>
+      <c r="I9" t="inlineStr">
+        <is>
+          <t>Extern gevoed synchroon met machine 110-240V AC (art. 1448)</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>1447</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>Dispensers (Vet)</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>Pulsarlube MSP DC (60 ml)</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>60 ml</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>Extern gevoed DC</t>
+        </is>
+      </c>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>G 3/8" M (of adapter 1/8" NPT)</t>
+        </is>
+      </c>
+      <c r="H10" t="inlineStr">
+        <is>
+          <t>Kunststof / RVS (IP65)</t>
+        </is>
+      </c>
+      <c r="I10" t="inlineStr">
+        <is>
+          <t>Extern gevoed synchroon met machine 12-24V DC (art. 1447)</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>1446</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>Dispensers (Vet)</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>Pulsarlube MSP AC (125 ml)</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>125 ml</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>Extern gevoed AC</t>
+        </is>
+      </c>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>G 3/8" M (of adapter 1/8" NPT)</t>
+        </is>
+      </c>
+      <c r="H11" t="inlineStr">
+        <is>
+          <t>Kunststof / RVS (IP65)</t>
+        </is>
+      </c>
+      <c r="I11" t="inlineStr">
+        <is>
+          <t>Extern gevoed synchroon met machine 110-240V AC (art. 1446)</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>1445</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>Dispensers (Vet)</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>Pulsarlube MSP DC (125 ml)</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>125 ml</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>Extern gevoed DC</t>
+        </is>
+      </c>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>G 3/8" M (of adapter 1/8" NPT)</t>
+        </is>
+      </c>
+      <c r="H12" t="inlineStr">
+        <is>
+          <t>Kunststof / RVS (IP65)</t>
+        </is>
+      </c>
+      <c r="I12" t="inlineStr">
+        <is>
+          <t>Extern gevoed synchroon met machine 12-24V DC (art. 1445)</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>1444</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>Dispensers (Vet)</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>Pulsarlube MSP AC (250 ml)</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>250 ml</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>Extern gevoed AC</t>
+        </is>
+      </c>
+      <c r="G13" t="inlineStr">
+        <is>
+          <t>G 3/8" M (of adapter 1/8" NPT)</t>
+        </is>
+      </c>
+      <c r="H13" t="inlineStr">
+        <is>
+          <t>Kunststof / RVS (IP65)</t>
+        </is>
+      </c>
+      <c r="I13" t="inlineStr">
+        <is>
+          <t>Extern gevoed synchroon met machine 110-240V AC (art. 1444)</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>1443</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>Dispensers (Vet)</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>Pulsarlube MSP DC (250 ml)</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>250 ml</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>Extern gevoed DC</t>
+        </is>
+      </c>
+      <c r="G14" t="inlineStr">
+        <is>
+          <t>G 3/8" M (of adapter 1/8" NPT)</t>
+        </is>
+      </c>
+      <c r="H14" t="inlineStr">
+        <is>
+          <t>Kunststof / RVS (IP65)</t>
+        </is>
+      </c>
+      <c r="I14" t="inlineStr">
+        <is>
+          <t>Extern gevoed synchroon met machine 12-24V DC (art. 1443)</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>1442</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>Dispensers (Vet)</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>Pulsarlube MSP AC (500 ml)</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>500 ml</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>Extern gevoed AC</t>
+        </is>
+      </c>
+      <c r="G15" t="inlineStr">
+        <is>
+          <t>G 3/8" M (of adapter 1/8" NPT)</t>
+        </is>
+      </c>
+      <c r="H15" t="inlineStr">
+        <is>
+          <t>Kunststof / RVS (IP65)</t>
+        </is>
+      </c>
+      <c r="I15" t="inlineStr">
+        <is>
+          <t>Extern gevoed synchroon met machine 110-240V AC (art. 1442)</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>1441</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>Dispensers (Vet)</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>Pulsarlube MSP DC (500 ml)</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>500 ml</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>Extern gevoed DC</t>
+        </is>
+      </c>
+      <c r="G16" t="inlineStr">
+        <is>
+          <t>G 3/8" M (of adapter 1/8" NPT)</t>
+        </is>
+      </c>
+      <c r="H16" t="inlineStr">
+        <is>
+          <t>Kunststof / RVS (IP65)</t>
+        </is>
+      </c>
+      <c r="I16" t="inlineStr">
+        <is>
+          <t>Extern gevoed synchroon met machine 12-24V DC (art. 1441)</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>1450</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>Dispensers (Vet)</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>Pulsarlube PLC monthly (60 ml)</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>60 ml</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>PLC gestuurd</t>
+        </is>
+      </c>
+      <c r="G17" t="inlineStr">
+        <is>
+          <t>G 3/8" M (of adapter 1/8" NPT)</t>
+        </is>
+      </c>
+      <c r="H17" t="inlineStr">
+        <is>
+          <t>Kunststof / RVS (IP65)</t>
+        </is>
+      </c>
+      <c r="I17" t="inlineStr">
+        <is>
+          <t>Aangestuurd via PLC signaal machine (art. 1450)</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>1455</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>Dispensers (Vet)</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>Pulsarlube PLC monthly (120 ml)</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>120 ml</t>
+        </is>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F18" t="inlineStr">
+        <is>
+          <t>PLC gestuurd</t>
+        </is>
+      </c>
+      <c r="G18" t="inlineStr">
+        <is>
+          <t>G 3/8" M (of adapter 1/8" NPT)</t>
+        </is>
+      </c>
+      <c r="H18" t="inlineStr">
+        <is>
+          <t>Kunststof / RVS (IP65)</t>
+        </is>
+      </c>
+      <c r="I18" t="inlineStr">
+        <is>
+          <t>Aangestuurd via PLC signaal machine (art. 1455)</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>1457</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>Dispensers (Vet)</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>Pulsarlube PLC monthly (240 ml)</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>240 ml</t>
+        </is>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F19" t="inlineStr">
+        <is>
+          <t>PLC gestuurd</t>
+        </is>
+      </c>
+      <c r="G19" t="inlineStr">
+        <is>
+          <t>G 3/8" M (of adapter 1/8" NPT)</t>
+        </is>
+      </c>
+      <c r="H19" t="inlineStr">
+        <is>
+          <t>Kunststof / RVS (IP65)</t>
+        </is>
+      </c>
+      <c r="I19" t="inlineStr">
+        <is>
+          <t>Aangestuurd via PLC signaal machine (art. 1457)</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>1459</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>Dispensers (Vet)</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>Pulsarlube PLC monthly (500 ml)</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>500 ml</t>
+        </is>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F20" t="inlineStr">
+        <is>
+          <t>PLC gestuurd</t>
+        </is>
+      </c>
+      <c r="G20" t="inlineStr">
+        <is>
+          <t>G 3/8" M (of adapter 1/8" NPT)</t>
+        </is>
+      </c>
+      <c r="H20" t="inlineStr">
+        <is>
+          <t>Kunststof / RVS (IP65)</t>
+        </is>
+      </c>
+      <c r="I20" t="inlineStr">
+        <is>
+          <t>Aangestuurd via PLC signaal machine (art. 1459)</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>1411</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>Dispensers (Olie)</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>Pulsarlube OL500 (500 ml)</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>500 ml</t>
+        </is>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>Olie</t>
+        </is>
+      </c>
+      <c r="F21" t="inlineStr">
+        <is>
+          <t>Oliedispenser herbruikbaar</t>
+        </is>
+      </c>
+      <c r="G21" t="inlineStr">
+        <is>
+          <t>1/8" NPT M</t>
+        </is>
+      </c>
+      <c r="H21" t="inlineStr">
+        <is>
+          <t>Kunststof / RVS</t>
+        </is>
+      </c>
+      <c r="I21" t="inlineStr">
+        <is>
+          <t>Elektro-mechanische oliesmeerdispenser 500 ml (art. 1411)</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>1437</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>Dispensers (Olie)</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>Pulsarlube MSP Oil AC (500 ml)</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>500 ml</t>
+        </is>
+      </c>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>Olie</t>
+        </is>
+      </c>
+      <c r="F22" t="inlineStr">
+        <is>
+          <t>Extern gevoed AC</t>
+        </is>
+      </c>
+      <c r="G22" t="inlineStr">
+        <is>
+          <t>1/8" NPT M</t>
+        </is>
+      </c>
+      <c r="H22" t="inlineStr">
+        <is>
+          <t>Kunststof / RVS</t>
+        </is>
+      </c>
+      <c r="I22" t="inlineStr">
+        <is>
+          <t>Oliesmeerdispenser extern gevoed 110-240V AC (art. 1437)</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>1449</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>Dispensers (Olie)</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>Pulsarlube MSP Oil DC (500 ml)</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>500 ml</t>
+        </is>
+      </c>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>Olie</t>
+        </is>
+      </c>
+      <c r="F23" t="inlineStr">
+        <is>
+          <t>Extern gevoed DC</t>
+        </is>
+      </c>
+      <c r="G23" t="inlineStr">
+        <is>
+          <t>1/8" NPT M</t>
+        </is>
+      </c>
+      <c r="H23" t="inlineStr">
+        <is>
+          <t>Kunststof / RVS</t>
+        </is>
+      </c>
+      <c r="I23" t="inlineStr">
+        <is>
+          <t>Oliesmeerdispenser extern gevoed 12-24V DC (art. 1449)</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>4419</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>Service Packs (Vetbalg + Batterij)</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>Servicepack + Grease MP2/3</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>60 ml</t>
+        </is>
+      </c>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>Grease MP2/3</t>
+        </is>
+      </c>
+      <c r="F24" t="inlineStr">
+        <is>
+          <t>Vervangbare balg</t>
+        </is>
+      </c>
+      <c r="G24" t="inlineStr">
+        <is>
+          <t>Pulsarlube bajonetsluiting</t>
+        </is>
+      </c>
+      <c r="H24" t="inlineStr">
+        <is>
+          <t>Vetbalg + Alkaline/Lithium batterij</t>
+        </is>
+      </c>
+      <c r="I24" t="inlineStr">
+        <is>
+          <t>Complete navulset 60 ml gevuld met Interflon Grease MP2/3 inclusief nieuwe batterijpack (art. 4419)</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>4210</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>Service Packs (Vetbalg + Batterij)</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>Servicepack + Food grease LT2</t>
+        </is>
+      </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>60 ml</t>
+        </is>
+      </c>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>Food grease LT2</t>
+        </is>
+      </c>
+      <c r="F25" t="inlineStr">
+        <is>
+          <t>Vervangbare balg</t>
+        </is>
+      </c>
+      <c r="G25" t="inlineStr">
+        <is>
+          <t>Pulsarlube bajonetsluiting</t>
+        </is>
+      </c>
+      <c r="H25" t="inlineStr">
+        <is>
+          <t>Vetbalg + Alkaline/Lithium batterij</t>
+        </is>
+      </c>
+      <c r="I25" t="inlineStr">
+        <is>
+          <t>Complete navulset 60 ml gevuld met Interflon Food grease LT2 inclusief nieuwe batterijpack (art. 4210)</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>4201</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>Service Packs (Vetbalg + Batterij)</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>Servicepack + Grease MP2/3</t>
+        </is>
+      </c>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>125 ml</t>
+        </is>
+      </c>
+      <c r="E26" t="inlineStr">
+        <is>
+          <t>Grease MP2/3</t>
+        </is>
+      </c>
+      <c r="F26" t="inlineStr">
+        <is>
+          <t>Vervangbare balg</t>
+        </is>
+      </c>
+      <c r="G26" t="inlineStr">
+        <is>
+          <t>Pulsarlube bajonetsluiting</t>
+        </is>
+      </c>
+      <c r="H26" t="inlineStr">
+        <is>
+          <t>Vetbalg + Alkaline/Lithium batterij</t>
+        </is>
+      </c>
+      <c r="I26" t="inlineStr">
+        <is>
+          <t>Complete navulset 125 ml gevuld met Interflon Grease MP2/3 inclusief nieuwe batterijpack (art. 4201)</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>4202</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>Service Packs (Vetbalg + Batterij)</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>Servicepack + Grease MP00</t>
+        </is>
+      </c>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>125 ml</t>
+        </is>
+      </c>
+      <c r="E27" t="inlineStr">
+        <is>
+          <t>Grease MP00</t>
+        </is>
+      </c>
+      <c r="F27" t="inlineStr">
+        <is>
+          <t>Vervangbare balg</t>
+        </is>
+      </c>
+      <c r="G27" t="inlineStr">
+        <is>
+          <t>Pulsarlube bajonetsluiting</t>
+        </is>
+      </c>
+      <c r="H27" t="inlineStr">
+        <is>
+          <t>Vetbalg + Alkaline/Lithium batterij</t>
+        </is>
+      </c>
+      <c r="I27" t="inlineStr">
+        <is>
+          <t>Complete navulset 125 ml gevuld met Interflon Grease MP00 inclusief nieuwe batterijpack (art. 4202)</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>4203</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>Service Packs (Vetbalg + Batterij)</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>Servicepack + Grease LS2</t>
+        </is>
+      </c>
+      <c r="D28" t="inlineStr">
+        <is>
+          <t>125 ml</t>
+        </is>
+      </c>
+      <c r="E28" t="inlineStr">
+        <is>
+          <t>Grease LS2</t>
+        </is>
+      </c>
+      <c r="F28" t="inlineStr">
+        <is>
+          <t>Vervangbare balg</t>
+        </is>
+      </c>
+      <c r="G28" t="inlineStr">
+        <is>
+          <t>Pulsarlube bajonetsluiting</t>
+        </is>
+      </c>
+      <c r="H28" t="inlineStr">
+        <is>
+          <t>Vetbalg + Alkaline/Lithium batterij</t>
+        </is>
+      </c>
+      <c r="I28" t="inlineStr">
+        <is>
+          <t>Complete navulset 125 ml gevuld met Interflon Grease LS2 inclusief nieuwe batterijpack (art. 4203)</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>4207</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>Service Packs (Vetbalg + Batterij)</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>Servicepack + Grease LS1/2</t>
+        </is>
+      </c>
+      <c r="D29" t="inlineStr">
+        <is>
+          <t>125 ml</t>
+        </is>
+      </c>
+      <c r="E29" t="inlineStr">
+        <is>
+          <t>Grease LS1/2</t>
+        </is>
+      </c>
+      <c r="F29" t="inlineStr">
+        <is>
+          <t>Vervangbare balg</t>
+        </is>
+      </c>
+      <c r="G29" t="inlineStr">
+        <is>
+          <t>Pulsarlube bajonetsluiting</t>
+        </is>
+      </c>
+      <c r="H29" t="inlineStr">
+        <is>
+          <t>Vetbalg + Alkaline/Lithium batterij</t>
+        </is>
+      </c>
+      <c r="I29" t="inlineStr">
+        <is>
+          <t>Complete navulset 125 ml gevuld met Interflon Grease LS1/2 inclusief nieuwe batterijpack (art. 4207)</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>4206</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>Service Packs (Vetbalg + Batterij)</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>Servicepack + Grease HTG</t>
+        </is>
+      </c>
+      <c r="D30" t="inlineStr">
+        <is>
+          <t>125 ml</t>
+        </is>
+      </c>
+      <c r="E30" t="inlineStr">
+        <is>
+          <t>Grease HTG</t>
+        </is>
+      </c>
+      <c r="F30" t="inlineStr">
+        <is>
+          <t>Vervangbare balg</t>
+        </is>
+      </c>
+      <c r="G30" t="inlineStr">
+        <is>
+          <t>Pulsarlube bajonetsluiting</t>
+        </is>
+      </c>
+      <c r="H30" t="inlineStr">
+        <is>
+          <t>Vetbalg + Alkaline/Lithium batterij</t>
+        </is>
+      </c>
+      <c r="I30" t="inlineStr">
+        <is>
+          <t>Complete navulset 125 ml gevuld met Interflon Grease HTG inclusief nieuwe batterijpack (art. 4206)</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>4209</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>Service Packs (Vetbalg + Batterij)</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>Servicepack + Grease HD2</t>
+        </is>
+      </c>
+      <c r="D31" t="inlineStr">
+        <is>
+          <t>125 ml</t>
+        </is>
+      </c>
+      <c r="E31" t="inlineStr">
+        <is>
+          <t>Grease HD2</t>
+        </is>
+      </c>
+      <c r="F31" t="inlineStr">
+        <is>
+          <t>Vervangbare balg</t>
+        </is>
+      </c>
+      <c r="G31" t="inlineStr">
+        <is>
+          <t>Pulsarlube bajonetsluiting</t>
+        </is>
+      </c>
+      <c r="H31" t="inlineStr">
+        <is>
+          <t>Vetbalg + Alkaline/Lithium batterij</t>
+        </is>
+      </c>
+      <c r="I31" t="inlineStr">
+        <is>
+          <t>Complete navulset 125 ml gevuld met Interflon Grease HD2 inclusief nieuwe batterijpack (art. 4209)</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>4204</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>Service Packs (Vetbalg + Batterij)</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>Servicepack + Food grease 1</t>
+        </is>
+      </c>
+      <c r="D32" t="inlineStr">
+        <is>
+          <t>125 ml</t>
+        </is>
+      </c>
+      <c r="E32" t="inlineStr">
+        <is>
+          <t>Food grease 1</t>
+        </is>
+      </c>
+      <c r="F32" t="inlineStr">
+        <is>
+          <t>Vervangbare balg</t>
+        </is>
+      </c>
+      <c r="G32" t="inlineStr">
+        <is>
+          <t>Pulsarlube bajonetsluiting</t>
+        </is>
+      </c>
+      <c r="H32" t="inlineStr">
+        <is>
+          <t>Vetbalg + Alkaline/Lithium batterij</t>
+        </is>
+      </c>
+      <c r="I32" t="inlineStr">
+        <is>
+          <t>Complete navulset 125 ml gevuld met Interflon Food grease 1 inclusief nieuwe batterijpack (art. 4204)</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>4205</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>Service Packs (Vetbalg + Batterij)</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>Servicepack + Food grease EP</t>
+        </is>
+      </c>
+      <c r="D33" t="inlineStr">
+        <is>
+          <t>125 ml</t>
+        </is>
+      </c>
+      <c r="E33" t="inlineStr">
+        <is>
+          <t>Food grease EP</t>
+        </is>
+      </c>
+      <c r="F33" t="inlineStr">
+        <is>
+          <t>Vervangbare balg</t>
+        </is>
+      </c>
+      <c r="G33" t="inlineStr">
+        <is>
+          <t>Pulsarlube bajonetsluiting</t>
+        </is>
+      </c>
+      <c r="H33" t="inlineStr">
+        <is>
+          <t>Vetbalg + Alkaline/Lithium batterij</t>
+        </is>
+      </c>
+      <c r="I33" t="inlineStr">
+        <is>
+          <t>Complete navulset 125 ml gevuld met Interflon Food grease EP inclusief nieuwe batterijpack (art. 4205)</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>4208</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>Service Packs (Vetbalg + Batterij)</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>Servicepack + Food grease LT2</t>
+        </is>
+      </c>
+      <c r="D34" t="inlineStr">
+        <is>
+          <t>125 ml</t>
+        </is>
+      </c>
+      <c r="E34" t="inlineStr">
+        <is>
+          <t>Food grease LT2</t>
+        </is>
+      </c>
+      <c r="F34" t="inlineStr">
+        <is>
+          <t>Vervangbare balg</t>
+        </is>
+      </c>
+      <c r="G34" t="inlineStr">
+        <is>
+          <t>Pulsarlube bajonetsluiting</t>
+        </is>
+      </c>
+      <c r="H34" t="inlineStr">
+        <is>
+          <t>Vetbalg + Alkaline/Lithium batterij</t>
+        </is>
+      </c>
+      <c r="I34" t="inlineStr">
+        <is>
+          <t>Complete navulset 125 ml gevuld met Interflon Food grease LT2 inclusief nieuwe batterijpack (art. 4208)</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>4401</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>Service Packs (Vetbalg + Batterij)</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>Servicepack + Grease MP2/3</t>
+        </is>
+      </c>
+      <c r="D35" t="inlineStr">
+        <is>
+          <t>250 ml</t>
+        </is>
+      </c>
+      <c r="E35" t="inlineStr">
+        <is>
+          <t>Grease MP2/3</t>
+        </is>
+      </c>
+      <c r="F35" t="inlineStr">
+        <is>
+          <t>Vervangbare balg</t>
+        </is>
+      </c>
+      <c r="G35" t="inlineStr">
+        <is>
+          <t>Pulsarlube bajonetsluiting</t>
+        </is>
+      </c>
+      <c r="H35" t="inlineStr">
+        <is>
+          <t>Vetbalg + Alkaline/Lithium batterij</t>
+        </is>
+      </c>
+      <c r="I35" t="inlineStr">
+        <is>
+          <t>Complete navulset 250 ml gevuld met Interflon Grease MP2/3 inclusief nieuwe batterijpack (art. 4401)</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>4402</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>Service Packs (Vetbalg + Batterij)</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>Servicepack + Grease MP1</t>
+        </is>
+      </c>
+      <c r="D36" t="inlineStr">
+        <is>
+          <t>250 ml</t>
+        </is>
+      </c>
+      <c r="E36" t="inlineStr">
+        <is>
+          <t>Grease MP1</t>
+        </is>
+      </c>
+      <c r="F36" t="inlineStr">
+        <is>
+          <t>Vervangbare balg</t>
+        </is>
+      </c>
+      <c r="G36" t="inlineStr">
+        <is>
+          <t>Pulsarlube bajonetsluiting</t>
+        </is>
+      </c>
+      <c r="H36" t="inlineStr">
+        <is>
+          <t>Vetbalg + Alkaline/Lithium batterij</t>
+        </is>
+      </c>
+      <c r="I36" t="inlineStr">
+        <is>
+          <t>Complete navulset 250 ml gevuld met Interflon Grease MP1 inclusief nieuwe batterijpack (art. 4402)</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>4403</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>Service Packs (Vetbalg + Batterij)</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>Servicepack + Grease LS2</t>
+        </is>
+      </c>
+      <c r="D37" t="inlineStr">
+        <is>
+          <t>250 ml</t>
+        </is>
+      </c>
+      <c r="E37" t="inlineStr">
+        <is>
+          <t>Grease LS2</t>
+        </is>
+      </c>
+      <c r="F37" t="inlineStr">
+        <is>
+          <t>Vervangbare balg</t>
+        </is>
+      </c>
+      <c r="G37" t="inlineStr">
+        <is>
+          <t>Pulsarlube bajonetsluiting</t>
+        </is>
+      </c>
+      <c r="H37" t="inlineStr">
+        <is>
+          <t>Vetbalg + Alkaline/Lithium batterij</t>
+        </is>
+      </c>
+      <c r="I37" t="inlineStr">
+        <is>
+          <t>Complete navulset 250 ml gevuld met Interflon Grease LS2 inclusief nieuwe batterijpack (art. 4403)</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>4407</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>Service Packs (Vetbalg + Batterij)</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>Servicepack + Grease LS1/2</t>
+        </is>
+      </c>
+      <c r="D38" t="inlineStr">
+        <is>
+          <t>250 ml</t>
+        </is>
+      </c>
+      <c r="E38" t="inlineStr">
+        <is>
+          <t>Grease LS1/2</t>
+        </is>
+      </c>
+      <c r="F38" t="inlineStr">
+        <is>
+          <t>Vervangbare balg</t>
+        </is>
+      </c>
+      <c r="G38" t="inlineStr">
+        <is>
+          <t>Pulsarlube bajonetsluiting</t>
+        </is>
+      </c>
+      <c r="H38" t="inlineStr">
+        <is>
+          <t>Vetbalg + Alkaline/Lithium batterij</t>
+        </is>
+      </c>
+      <c r="I38" t="inlineStr">
+        <is>
+          <t>Complete navulset 250 ml gevuld met Interflon Grease LS1/2 inclusief nieuwe batterijpack (art. 4407)</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>4406</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>Service Packs (Vetbalg + Batterij)</t>
+        </is>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>Servicepack + Grease HTG</t>
+        </is>
+      </c>
+      <c r="D39" t="inlineStr">
+        <is>
+          <t>250 ml</t>
+        </is>
+      </c>
+      <c r="E39" t="inlineStr">
+        <is>
+          <t>Grease HTG</t>
+        </is>
+      </c>
+      <c r="F39" t="inlineStr">
+        <is>
+          <t>Vervangbare balg</t>
+        </is>
+      </c>
+      <c r="G39" t="inlineStr">
+        <is>
+          <t>Pulsarlube bajonetsluiting</t>
+        </is>
+      </c>
+      <c r="H39" t="inlineStr">
+        <is>
+          <t>Vetbalg + Alkaline/Lithium batterij</t>
+        </is>
+      </c>
+      <c r="I39" t="inlineStr">
+        <is>
+          <t>Complete navulset 250 ml gevuld met Interflon Grease HTG inclusief nieuwe batterijpack (art. 4406)</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>4418</t>
+        </is>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>Service Packs (Vetbalg + Batterij)</t>
+        </is>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>Servicepack + Grease HD2</t>
+        </is>
+      </c>
+      <c r="D40" t="inlineStr">
+        <is>
+          <t>250 ml</t>
+        </is>
+      </c>
+      <c r="E40" t="inlineStr">
+        <is>
+          <t>Grease HD2</t>
+        </is>
+      </c>
+      <c r="F40" t="inlineStr">
+        <is>
+          <t>Vervangbare balg</t>
+        </is>
+      </c>
+      <c r="G40" t="inlineStr">
+        <is>
+          <t>Pulsarlube bajonetsluiting</t>
+        </is>
+      </c>
+      <c r="H40" t="inlineStr">
+        <is>
+          <t>Vetbalg + Alkaline/Lithium batterij</t>
+        </is>
+      </c>
+      <c r="I40" t="inlineStr">
+        <is>
+          <t>Complete navulset 250 ml gevuld met Interflon Grease HD2 inclusief nieuwe batterijpack (art. 4418)</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>4404</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>Service Packs (Vetbalg + Batterij)</t>
+        </is>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>Servicepack + Food grease 1</t>
+        </is>
+      </c>
+      <c r="D41" t="inlineStr">
+        <is>
+          <t>250 ml</t>
+        </is>
+      </c>
+      <c r="E41" t="inlineStr">
+        <is>
+          <t>Food grease 1</t>
+        </is>
+      </c>
+      <c r="F41" t="inlineStr">
+        <is>
+          <t>Vervangbare balg</t>
+        </is>
+      </c>
+      <c r="G41" t="inlineStr">
+        <is>
+          <t>Pulsarlube bajonetsluiting</t>
+        </is>
+      </c>
+      <c r="H41" t="inlineStr">
+        <is>
+          <t>Vetbalg + Alkaline/Lithium batterij</t>
+        </is>
+      </c>
+      <c r="I41" t="inlineStr">
+        <is>
+          <t>Complete navulset 250 ml gevuld met Interflon Food grease 1 inclusief nieuwe batterijpack (art. 4404)</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>4405</t>
+        </is>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>Service Packs (Vetbalg + Batterij)</t>
+        </is>
+      </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>Servicepack + Food grease EP</t>
+        </is>
+      </c>
+      <c r="D42" t="inlineStr">
+        <is>
+          <t>250 ml</t>
+        </is>
+      </c>
+      <c r="E42" t="inlineStr">
+        <is>
+          <t>Food grease EP</t>
+        </is>
+      </c>
+      <c r="F42" t="inlineStr">
+        <is>
+          <t>Vervangbare balg</t>
+        </is>
+      </c>
+      <c r="G42" t="inlineStr">
+        <is>
+          <t>Pulsarlube bajonetsluiting</t>
+        </is>
+      </c>
+      <c r="H42" t="inlineStr">
+        <is>
+          <t>Vetbalg + Alkaline/Lithium batterij</t>
+        </is>
+      </c>
+      <c r="I42" t="inlineStr">
+        <is>
+          <t>Complete navulset 250 ml gevuld met Interflon Food grease EP inclusief nieuwe batterijpack (art. 4405)</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>4415</t>
+        </is>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>Service Packs (Vetbalg + Batterij)</t>
+        </is>
+      </c>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>Servicepack + Food grease LT2</t>
+        </is>
+      </c>
+      <c r="D43" t="inlineStr">
+        <is>
+          <t>250 ml</t>
+        </is>
+      </c>
+      <c r="E43" t="inlineStr">
+        <is>
+          <t>Food grease LT2</t>
+        </is>
+      </c>
+      <c r="F43" t="inlineStr">
+        <is>
+          <t>Vervangbare balg</t>
+        </is>
+      </c>
+      <c r="G43" t="inlineStr">
+        <is>
+          <t>Pulsarlube bajonetsluiting</t>
+        </is>
+      </c>
+      <c r="H43" t="inlineStr">
+        <is>
+          <t>Vetbalg + Alkaline/Lithium batterij</t>
+        </is>
+      </c>
+      <c r="I43" t="inlineStr">
+        <is>
+          <t>Complete navulset 250 ml gevuld met Interflon Food grease LT2 inclusief nieuwe batterijpack (art. 4415)</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>4408</t>
+        </is>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>Service Packs (Vetbalg + Batterij)</t>
+        </is>
+      </c>
+      <c r="C44" t="inlineStr">
+        <is>
+          <t>Servicepack + Grease MP2/3</t>
+        </is>
+      </c>
+      <c r="D44" t="inlineStr">
+        <is>
+          <t>500 ml</t>
+        </is>
+      </c>
+      <c r="E44" t="inlineStr">
+        <is>
+          <t>Grease MP2/3</t>
+        </is>
+      </c>
+      <c r="F44" t="inlineStr">
+        <is>
+          <t>Vervangbare balg</t>
+        </is>
+      </c>
+      <c r="G44" t="inlineStr">
+        <is>
+          <t>Pulsarlube bajonetsluiting</t>
+        </is>
+      </c>
+      <c r="H44" t="inlineStr">
+        <is>
+          <t>Vetbalg + Alkaline/Lithium batterij</t>
+        </is>
+      </c>
+      <c r="I44" t="inlineStr">
+        <is>
+          <t>Complete navulset 500 ml gevuld met Interflon Grease MP2/3 inclusief nieuwe batterijpack (art. 4408)</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>4426</t>
+        </is>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>Service Packs (Vetbalg + Batterij)</t>
+        </is>
+      </c>
+      <c r="C45" t="inlineStr">
+        <is>
+          <t>Servicepack + Grease MP1</t>
+        </is>
+      </c>
+      <c r="D45" t="inlineStr">
+        <is>
+          <t>500 ml</t>
+        </is>
+      </c>
+      <c r="E45" t="inlineStr">
+        <is>
+          <t>Grease MP1</t>
+        </is>
+      </c>
+      <c r="F45" t="inlineStr">
+        <is>
+          <t>Vervangbare balg</t>
+        </is>
+      </c>
+      <c r="G45" t="inlineStr">
+        <is>
+          <t>Pulsarlube bajonetsluiting</t>
+        </is>
+      </c>
+      <c r="H45" t="inlineStr">
+        <is>
+          <t>Vetbalg + Alkaline/Lithium batterij</t>
+        </is>
+      </c>
+      <c r="I45" t="inlineStr">
+        <is>
+          <t>Complete navulset 500 ml gevuld met Interflon Grease MP1 inclusief nieuwe batterijpack (art. 4426)</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>4409</t>
+        </is>
+      </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>Service Packs (Vetbalg + Batterij)</t>
+        </is>
+      </c>
+      <c r="C46" t="inlineStr">
+        <is>
+          <t>Servicepack + Grease LS2</t>
+        </is>
+      </c>
+      <c r="D46" t="inlineStr">
+        <is>
+          <t>500 ml</t>
+        </is>
+      </c>
+      <c r="E46" t="inlineStr">
+        <is>
+          <t>Grease LS2</t>
+        </is>
+      </c>
+      <c r="F46" t="inlineStr">
+        <is>
+          <t>Vervangbare balg</t>
+        </is>
+      </c>
+      <c r="G46" t="inlineStr">
+        <is>
+          <t>Pulsarlube bajonetsluiting</t>
+        </is>
+      </c>
+      <c r="H46" t="inlineStr">
+        <is>
+          <t>Vetbalg + Alkaline/Lithium batterij</t>
+        </is>
+      </c>
+      <c r="I46" t="inlineStr">
+        <is>
+          <t>Complete navulset 500 ml gevuld met Interflon Grease LS2 inclusief nieuwe batterijpack (art. 4409)</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>4413</t>
+        </is>
+      </c>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>Service Packs (Vetbalg + Batterij)</t>
+        </is>
+      </c>
+      <c r="C47" t="inlineStr">
+        <is>
+          <t>Servicepack + Grease LS1/2</t>
+        </is>
+      </c>
+      <c r="D47" t="inlineStr">
+        <is>
+          <t>500 ml</t>
+        </is>
+      </c>
+      <c r="E47" t="inlineStr">
+        <is>
+          <t>Grease LS1/2</t>
+        </is>
+      </c>
+      <c r="F47" t="inlineStr">
+        <is>
+          <t>Vervangbare balg</t>
+        </is>
+      </c>
+      <c r="G47" t="inlineStr">
+        <is>
+          <t>Pulsarlube bajonetsluiting</t>
+        </is>
+      </c>
+      <c r="H47" t="inlineStr">
+        <is>
+          <t>Vetbalg + Alkaline/Lithium batterij</t>
+        </is>
+      </c>
+      <c r="I47" t="inlineStr">
+        <is>
+          <t>Complete navulset 500 ml gevuld met Interflon Grease LS1/2 inclusief nieuwe batterijpack (art. 4413)</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>4412</t>
+        </is>
+      </c>
+      <c r="B48" t="inlineStr">
+        <is>
+          <t>Service Packs (Vetbalg + Batterij)</t>
+        </is>
+      </c>
+      <c r="C48" t="inlineStr">
+        <is>
+          <t>Servicepack + Grease HTG</t>
+        </is>
+      </c>
+      <c r="D48" t="inlineStr">
+        <is>
+          <t>500 ml</t>
+        </is>
+      </c>
+      <c r="E48" t="inlineStr">
+        <is>
+          <t>Grease HTG</t>
+        </is>
+      </c>
+      <c r="F48" t="inlineStr">
+        <is>
+          <t>Vervangbare balg</t>
+        </is>
+      </c>
+      <c r="G48" t="inlineStr">
+        <is>
+          <t>Pulsarlube bajonetsluiting</t>
+        </is>
+      </c>
+      <c r="H48" t="inlineStr">
+        <is>
+          <t>Vetbalg + Alkaline/Lithium batterij</t>
+        </is>
+      </c>
+      <c r="I48" t="inlineStr">
+        <is>
+          <t>Complete navulset 500 ml gevuld met Interflon Grease HTG inclusief nieuwe batterijpack (art. 4412)</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>4416</t>
+        </is>
+      </c>
+      <c r="B49" t="inlineStr">
+        <is>
+          <t>Service Packs (Vetbalg + Batterij)</t>
+        </is>
+      </c>
+      <c r="C49" t="inlineStr">
+        <is>
+          <t>Servicepack + Grease HD2</t>
+        </is>
+      </c>
+      <c r="D49" t="inlineStr">
+        <is>
+          <t>500 ml</t>
+        </is>
+      </c>
+      <c r="E49" t="inlineStr">
+        <is>
+          <t>Grease HD2</t>
+        </is>
+      </c>
+      <c r="F49" t="inlineStr">
+        <is>
+          <t>Vervangbare balg</t>
+        </is>
+      </c>
+      <c r="G49" t="inlineStr">
+        <is>
+          <t>Pulsarlube bajonetsluiting</t>
+        </is>
+      </c>
+      <c r="H49" t="inlineStr">
+        <is>
+          <t>Vetbalg + Alkaline/Lithium batterij</t>
+        </is>
+      </c>
+      <c r="I49" t="inlineStr">
+        <is>
+          <t>Complete navulset 500 ml gevuld met Interflon Grease HD2 inclusief nieuwe batterijpack (art. 4416)</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="inlineStr">
+        <is>
+          <t>4424</t>
+        </is>
+      </c>
+      <c r="B50" t="inlineStr">
+        <is>
+          <t>Service Packs (Vetbalg + Batterij)</t>
+        </is>
+      </c>
+      <c r="C50" t="inlineStr">
+        <is>
+          <t>Servicepack + Grease HS2</t>
+        </is>
+      </c>
+      <c r="D50" t="inlineStr">
+        <is>
+          <t>500 ml</t>
+        </is>
+      </c>
+      <c r="E50" t="inlineStr">
+        <is>
+          <t>Grease HS2</t>
+        </is>
+      </c>
+      <c r="F50" t="inlineStr">
+        <is>
+          <t>Vervangbare balg</t>
+        </is>
+      </c>
+      <c r="G50" t="inlineStr">
+        <is>
+          <t>Pulsarlube bajonetsluiting</t>
+        </is>
+      </c>
+      <c r="H50" t="inlineStr">
+        <is>
+          <t>Vetbalg + Alkaline/Lithium batterij</t>
+        </is>
+      </c>
+      <c r="I50" t="inlineStr">
+        <is>
+          <t>Complete navulset 500 ml gevuld met Interflon Grease HS2 inclusief nieuwe batterijpack (art. 4424)</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="inlineStr">
+        <is>
+          <t>4410</t>
+        </is>
+      </c>
+      <c r="B51" t="inlineStr">
+        <is>
+          <t>Service Packs (Vetbalg + Batterij)</t>
+        </is>
+      </c>
+      <c r="C51" t="inlineStr">
+        <is>
+          <t>Servicepack + Food grease 1</t>
+        </is>
+      </c>
+      <c r="D51" t="inlineStr">
+        <is>
+          <t>500 ml</t>
+        </is>
+      </c>
+      <c r="E51" t="inlineStr">
+        <is>
+          <t>Food grease 1</t>
+        </is>
+      </c>
+      <c r="F51" t="inlineStr">
+        <is>
+          <t>Vervangbare balg</t>
+        </is>
+      </c>
+      <c r="G51" t="inlineStr">
+        <is>
+          <t>Pulsarlube bajonetsluiting</t>
+        </is>
+      </c>
+      <c r="H51" t="inlineStr">
+        <is>
+          <t>Vetbalg + Alkaline/Lithium batterij</t>
+        </is>
+      </c>
+      <c r="I51" t="inlineStr">
+        <is>
+          <t>Complete navulset 500 ml gevuld met Interflon Food grease 1 inclusief nieuwe batterijpack (art. 4410)</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="inlineStr">
+        <is>
+          <t>4411</t>
+        </is>
+      </c>
+      <c r="B52" t="inlineStr">
+        <is>
+          <t>Service Packs (Vetbalg + Batterij)</t>
+        </is>
+      </c>
+      <c r="C52" t="inlineStr">
+        <is>
+          <t>Servicepack + Food grease EP</t>
+        </is>
+      </c>
+      <c r="D52" t="inlineStr">
+        <is>
+          <t>500 ml</t>
+        </is>
+      </c>
+      <c r="E52" t="inlineStr">
+        <is>
+          <t>Food grease EP</t>
+        </is>
+      </c>
+      <c r="F52" t="inlineStr">
+        <is>
+          <t>Vervangbare balg</t>
+        </is>
+      </c>
+      <c r="G52" t="inlineStr">
+        <is>
+          <t>Pulsarlube bajonetsluiting</t>
+        </is>
+      </c>
+      <c r="H52" t="inlineStr">
+        <is>
+          <t>Vetbalg + Alkaline/Lithium batterij</t>
+        </is>
+      </c>
+      <c r="I52" t="inlineStr">
+        <is>
+          <t>Complete navulset 500 ml gevuld met Interflon Food grease EP inclusief nieuwe batterijpack (art. 4411)</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="inlineStr">
+        <is>
+          <t>4414</t>
+        </is>
+      </c>
+      <c r="B53" t="inlineStr">
+        <is>
+          <t>Service Packs (Vetbalg + Batterij)</t>
+        </is>
+      </c>
+      <c r="C53" t="inlineStr">
+        <is>
+          <t>Servicepack + Food grease LT2</t>
+        </is>
+      </c>
+      <c r="D53" t="inlineStr">
+        <is>
+          <t>500 ml</t>
+        </is>
+      </c>
+      <c r="E53" t="inlineStr">
+        <is>
+          <t>Food grease LT2</t>
+        </is>
+      </c>
+      <c r="F53" t="inlineStr">
+        <is>
+          <t>Vervangbare balg</t>
+        </is>
+      </c>
+      <c r="G53" t="inlineStr">
+        <is>
+          <t>Pulsarlube bajonetsluiting</t>
+        </is>
+      </c>
+      <c r="H53" t="inlineStr">
+        <is>
+          <t>Vetbalg + Alkaline/Lithium batterij</t>
+        </is>
+      </c>
+      <c r="I53" t="inlineStr">
+        <is>
+          <t>Complete navulset 500 ml gevuld met Interflon Food grease LT2 inclusief nieuwe batterijpack (art. 4414)</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="inlineStr">
+        <is>
+          <t>4425</t>
+        </is>
+      </c>
+      <c r="B54" t="inlineStr">
+        <is>
+          <t>Service Packs (Vetbalg + Batterij)</t>
+        </is>
+      </c>
+      <c r="C54" t="inlineStr">
+        <is>
+          <t>Servicepack + Food grease HD2</t>
+        </is>
+      </c>
+      <c r="D54" t="inlineStr">
+        <is>
+          <t>500 ml</t>
+        </is>
+      </c>
+      <c r="E54" t="inlineStr">
+        <is>
+          <t>Food grease HD2</t>
+        </is>
+      </c>
+      <c r="F54" t="inlineStr">
+        <is>
+          <t>Vervangbare balg</t>
+        </is>
+      </c>
+      <c r="G54" t="inlineStr">
+        <is>
+          <t>Pulsarlube bajonetsluiting</t>
+        </is>
+      </c>
+      <c r="H54" t="inlineStr">
+        <is>
+          <t>Vetbalg + Alkaline/Lithium batterij</t>
+        </is>
+      </c>
+      <c r="I54" t="inlineStr">
+        <is>
+          <t>Complete navulset 500 ml gevuld met Interflon Food grease HD2 inclusief nieuwe batterijpack (art. 4425)</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="inlineStr">
+        <is>
+          <t>4428</t>
+        </is>
+      </c>
+      <c r="B55" t="inlineStr">
+        <is>
+          <t>Service Packs (Vetbalg + Batterij)</t>
+        </is>
+      </c>
+      <c r="C55" t="inlineStr">
+        <is>
+          <t>Servicepack + Food grease HS1</t>
+        </is>
+      </c>
+      <c r="D55" t="inlineStr">
+        <is>
+          <t>500 ml</t>
+        </is>
+      </c>
+      <c r="E55" t="inlineStr">
+        <is>
+          <t>Food grease HS1</t>
+        </is>
+      </c>
+      <c r="F55" t="inlineStr">
+        <is>
+          <t>Vervangbare balg</t>
+        </is>
+      </c>
+      <c r="G55" t="inlineStr">
+        <is>
+          <t>Pulsarlube bajonetsluiting</t>
+        </is>
+      </c>
+      <c r="H55" t="inlineStr">
+        <is>
+          <t>Vetbalg + Alkaline/Lithium batterij</t>
+        </is>
+      </c>
+      <c r="I55" t="inlineStr">
+        <is>
+          <t>Complete navulset 500 ml gevuld met Interflon Food grease HS1 inclusief nieuwe batterijpack (art. 4428)</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="inlineStr">
+        <is>
+          <t>1480</t>
+        </is>
+      </c>
+      <c r="B56" t="inlineStr">
+        <is>
+          <t>Verdeelblokken</t>
+        </is>
+      </c>
+      <c r="C56" t="inlineStr">
+        <is>
+          <t>HU Type Divider Block 2 poorten</t>
+        </is>
+      </c>
+      <c r="D56" t="inlineStr">
+        <is>
+          <t>2 uitgangen</t>
+        </is>
+      </c>
+      <c r="E56" t="inlineStr">
+        <is>
+          <t>Vet</t>
+        </is>
+      </c>
+      <c r="F56" t="inlineStr">
+        <is>
+          <t>Inlaat 1/8" NPT F</t>
+        </is>
+      </c>
+      <c r="G56" t="inlineStr">
+        <is>
+          <t>2x Uitlaat 1/8" NPT F</t>
+        </is>
+      </c>
+      <c r="H56" t="inlineStr">
+        <is>
+          <t>Vernikkeld staal</t>
+        </is>
+      </c>
+      <c r="I56" t="inlineStr">
+        <is>
+          <t>Progressief verdeelblok 2 poorten voor Pulsarlube (max. 4m leiding) (art. 1480)</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="inlineStr">
+        <is>
+          <t>1481</t>
+        </is>
+      </c>
+      <c r="B57" t="inlineStr">
+        <is>
+          <t>Verdeelblokken</t>
+        </is>
+      </c>
+      <c r="C57" t="inlineStr">
+        <is>
+          <t>HU Type Divider Block 3 poorten</t>
+        </is>
+      </c>
+      <c r="D57" t="inlineStr">
+        <is>
+          <t>3 uitgangen</t>
+        </is>
+      </c>
+      <c r="E57" t="inlineStr">
+        <is>
+          <t>Vet</t>
+        </is>
+      </c>
+      <c r="F57" t="inlineStr">
+        <is>
+          <t>Inlaat 1/8" NPT F</t>
+        </is>
+      </c>
+      <c r="G57" t="inlineStr">
+        <is>
+          <t>3x Uitlaat 1/8" NPT F</t>
+        </is>
+      </c>
+      <c r="H57" t="inlineStr">
+        <is>
+          <t>Vernikkeld staal</t>
+        </is>
+      </c>
+      <c r="I57" t="inlineStr">
+        <is>
+          <t>Progressief verdeelblok 3 poorten voor Pulsarlube (max. 4m leiding) (art. 1481)</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="inlineStr">
+        <is>
+          <t>1482</t>
+        </is>
+      </c>
+      <c r="B58" t="inlineStr">
+        <is>
+          <t>Verdeelblokken</t>
+        </is>
+      </c>
+      <c r="C58" t="inlineStr">
+        <is>
+          <t>HU Type Divider Block 4 poorten</t>
+        </is>
+      </c>
+      <c r="D58" t="inlineStr">
+        <is>
+          <t>4 uitgangen</t>
+        </is>
+      </c>
+      <c r="E58" t="inlineStr">
+        <is>
+          <t>Vet</t>
+        </is>
+      </c>
+      <c r="F58" t="inlineStr">
+        <is>
+          <t>Inlaat 1/8" NPT F</t>
+        </is>
+      </c>
+      <c r="G58" t="inlineStr">
+        <is>
+          <t>4x Uitlaat 1/8" NPT F</t>
+        </is>
+      </c>
+      <c r="H58" t="inlineStr">
+        <is>
+          <t>Vernikkeld staal</t>
+        </is>
+      </c>
+      <c r="I58" t="inlineStr">
+        <is>
+          <t>Progressief verdeelblok 4 poorten voor Pulsarlube (max. 4m leiding) (art. 1482)</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="inlineStr">
+        <is>
+          <t>1483</t>
+        </is>
+      </c>
+      <c r="B59" t="inlineStr">
+        <is>
+          <t>Verdeelblokken</t>
+        </is>
+      </c>
+      <c r="C59" t="inlineStr">
+        <is>
+          <t>HU Type Divider Block 5 poorten</t>
+        </is>
+      </c>
+      <c r="D59" t="inlineStr">
+        <is>
+          <t>5 uitgangen</t>
+        </is>
+      </c>
+      <c r="E59" t="inlineStr">
+        <is>
+          <t>Vet</t>
+        </is>
+      </c>
+      <c r="F59" t="inlineStr">
+        <is>
+          <t>Inlaat 1/8" NPT F</t>
+        </is>
+      </c>
+      <c r="G59" t="inlineStr">
+        <is>
+          <t>5x Uitlaat 1/8" NPT F</t>
+        </is>
+      </c>
+      <c r="H59" t="inlineStr">
+        <is>
+          <t>Vernikkeld staal</t>
+        </is>
+      </c>
+      <c r="I59" t="inlineStr">
+        <is>
+          <t>Progressief verdeelblok 5 poorten voor Pulsarlube (max. 4m leiding) (art. 1483)</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" t="inlineStr">
+        <is>
+          <t>1484</t>
+        </is>
+      </c>
+      <c r="B60" t="inlineStr">
+        <is>
+          <t>Verdeelblokken</t>
+        </is>
+      </c>
+      <c r="C60" t="inlineStr">
+        <is>
+          <t>HU Type Divider Block 6 poorten</t>
+        </is>
+      </c>
+      <c r="D60" t="inlineStr">
+        <is>
+          <t>6 uitgangen</t>
+        </is>
+      </c>
+      <c r="E60" t="inlineStr">
+        <is>
+          <t>Vet</t>
+        </is>
+      </c>
+      <c r="F60" t="inlineStr">
+        <is>
+          <t>Inlaat 1/8" NPT F</t>
+        </is>
+      </c>
+      <c r="G60" t="inlineStr">
+        <is>
+          <t>6x Uitlaat 1/8" NPT F</t>
+        </is>
+      </c>
+      <c r="H60" t="inlineStr">
+        <is>
+          <t>Vernikkeld staal</t>
+        </is>
+      </c>
+      <c r="I60" t="inlineStr">
+        <is>
+          <t>Progressief verdeelblok 6 poorten voor Pulsarlube (max. 4m leiding) (art. 1484)</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" t="inlineStr">
+        <is>
+          <t>1485</t>
+        </is>
+      </c>
+      <c r="B61" t="inlineStr">
+        <is>
+          <t>Verdeelblokken</t>
+        </is>
+      </c>
+      <c r="C61" t="inlineStr">
+        <is>
+          <t>HU Type Divider Block 7 poorten</t>
+        </is>
+      </c>
+      <c r="D61" t="inlineStr">
+        <is>
+          <t>7 uitgangen</t>
+        </is>
+      </c>
+      <c r="E61" t="inlineStr">
+        <is>
+          <t>Vet</t>
+        </is>
+      </c>
+      <c r="F61" t="inlineStr">
+        <is>
+          <t>Inlaat 1/8" NPT F</t>
+        </is>
+      </c>
+      <c r="G61" t="inlineStr">
+        <is>
+          <t>7x Uitlaat 1/8" NPT F</t>
+        </is>
+      </c>
+      <c r="H61" t="inlineStr">
+        <is>
+          <t>Vernikkeld staal</t>
+        </is>
+      </c>
+      <c r="I61" t="inlineStr">
+        <is>
+          <t>Progressief verdeelblok 7 poorten voor Pulsarlube (max. 4m leiding) (art. 1485)</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" t="inlineStr">
+        <is>
+          <t>1486</t>
+        </is>
+      </c>
+      <c r="B62" t="inlineStr">
+        <is>
+          <t>Verdeelblokken</t>
+        </is>
+      </c>
+      <c r="C62" t="inlineStr">
+        <is>
+          <t>HU Type Divider Block 8 poorten</t>
+        </is>
+      </c>
+      <c r="D62" t="inlineStr">
+        <is>
+          <t>8 uitgangen</t>
+        </is>
+      </c>
+      <c r="E62" t="inlineStr">
+        <is>
+          <t>Vet</t>
+        </is>
+      </c>
+      <c r="F62" t="inlineStr">
+        <is>
+          <t>Inlaat 1/8" NPT F</t>
+        </is>
+      </c>
+      <c r="G62" t="inlineStr">
+        <is>
+          <t>8x Uitlaat 1/8" NPT F</t>
+        </is>
+      </c>
+      <c r="H62" t="inlineStr">
+        <is>
+          <t>Vernikkeld staal</t>
+        </is>
+      </c>
+      <c r="I62" t="inlineStr">
+        <is>
+          <t>Progressief verdeelblok 8 poorten voor Pulsarlube (max. 4m leiding) (art. 1486)</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" t="inlineStr">
+        <is>
+          <t>1475</t>
+        </is>
+      </c>
+      <c r="B63" t="inlineStr">
+        <is>
+          <t>Nylon Leidingen</t>
+        </is>
+      </c>
+      <c r="C63" t="inlineStr">
+        <is>
+          <t>Nylon tube 4 mm (per meter)</t>
+        </is>
+      </c>
+      <c r="D63" t="inlineStr">
+        <is>
+          <t>4 mm OD / 2.5 mm ID</t>
+        </is>
+      </c>
+      <c r="E63" t="inlineStr">
+        <is>
+          <t>Olie</t>
+        </is>
+      </c>
+      <c r="F63" t="inlineStr">
+        <is>
+          <t>Push-in 4 mm</t>
+        </is>
+      </c>
+      <c r="G63" t="inlineStr">
+        <is>
+          <t>Push-in 4 mm</t>
+        </is>
+      </c>
+      <c r="H63" t="inlineStr">
+        <is>
+          <t>Nylon PA12</t>
+        </is>
+      </c>
+      <c r="I63" t="inlineStr">
+        <is>
+          <t>Hogedrukleiding 4 mm voor Pulsarlube oliesmeersystemen (art. 1475)</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" t="inlineStr">
+        <is>
+          <t>1431</t>
+        </is>
+      </c>
+      <c r="B64" t="inlineStr">
+        <is>
+          <t>Nylon Leidingen</t>
+        </is>
+      </c>
+      <c r="C64" t="inlineStr">
+        <is>
+          <t>Nylon tube 6 mm (per meter)</t>
+        </is>
+      </c>
+      <c r="D64" t="inlineStr">
+        <is>
+          <t>6 mm OD / 4 mm ID</t>
+        </is>
+      </c>
+      <c r="E64" t="inlineStr">
+        <is>
+          <t>Vet / Olie</t>
+        </is>
+      </c>
+      <c r="F64" t="inlineStr">
+        <is>
+          <t>Push-in 6 mm</t>
+        </is>
+      </c>
+      <c r="G64" t="inlineStr">
+        <is>
+          <t>Push-in 6 mm</t>
+        </is>
+      </c>
+      <c r="H64" t="inlineStr">
+        <is>
+          <t>Nylon PA12</t>
+        </is>
+      </c>
+      <c r="I64" t="inlineStr">
+        <is>
+          <t>Hogedrukleiding 6 mm voor Pulsarlube verdeelblokken en installatiekits (art. 1431)</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" t="inlineStr">
+        <is>
+          <t>1706</t>
+        </is>
+      </c>
+      <c r="B65" t="inlineStr">
+        <is>
+          <t>Nylon Leidingen</t>
+        </is>
+      </c>
+      <c r="C65" t="inlineStr">
+        <is>
+          <t>Nylon tube 8 mm (per meter)</t>
+        </is>
+      </c>
+      <c r="D65" t="inlineStr">
+        <is>
+          <t>8 mm OD / 6 mm ID</t>
+        </is>
+      </c>
+      <c r="E65" t="inlineStr">
+        <is>
+          <t>Vet</t>
+        </is>
+      </c>
+      <c r="F65" t="inlineStr">
+        <is>
+          <t>Push-in 8 mm</t>
+        </is>
+      </c>
+      <c r="G65" t="inlineStr">
+        <is>
+          <t>Push-in 8 mm</t>
+        </is>
+      </c>
+      <c r="H65" t="inlineStr">
+        <is>
+          <t>Nylon PA12</t>
+        </is>
+      </c>
+      <c r="I65" t="inlineStr">
+        <is>
+          <t>Hogedrukleiding 8 mm voor Pulsarlube vetinstallatiekits tot 4m (art. 1706)</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" t="inlineStr">
+        <is>
+          <t>1413</t>
+        </is>
+      </c>
+      <c r="B66" t="inlineStr">
+        <is>
+          <t>Borstelsets</t>
+        </is>
+      </c>
+      <c r="C66" t="inlineStr">
+        <is>
+          <t>Borstelkit 2" plat nylon (1/8" NPT)</t>
+        </is>
+      </c>
+      <c r="D66" t="inlineStr">
+        <is>
+          <t>2 inch (50 mm)</t>
+        </is>
+      </c>
+      <c r="E66" t="inlineStr">
+        <is>
+          <t>Olie / Vet</t>
+        </is>
+      </c>
+      <c r="F66" t="inlineStr">
+        <is>
+          <t>1/8" NPT F</t>
+        </is>
+      </c>
+      <c r="G66" t="inlineStr">
+        <is>
+          <t>Platte borstel nylon</t>
+        </is>
+      </c>
+      <c r="H66" t="inlineStr">
+        <is>
+          <t>Messing / Nylon borstelharen</t>
+        </is>
+      </c>
+      <c r="I66" t="inlineStr">
+        <is>
+          <t>Platte kettingsmeerborstel 2 inch inclusief montagebeugel en doorvoer (art. 1413)</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" t="inlineStr">
+        <is>
+          <t>1414</t>
+        </is>
+      </c>
+      <c r="B67" t="inlineStr">
+        <is>
+          <t>Borstelsets</t>
+        </is>
+      </c>
+      <c r="C67" t="inlineStr">
+        <is>
+          <t>Borstelkit 1" rond nylon (1/8" NPT)</t>
+        </is>
+      </c>
+      <c r="D67" t="inlineStr">
+        <is>
+          <t>1 inch (25 mm)</t>
+        </is>
+      </c>
+      <c r="E67" t="inlineStr">
+        <is>
+          <t>Olie / Vet</t>
+        </is>
+      </c>
+      <c r="F67" t="inlineStr">
+        <is>
+          <t>1/8" NPT F</t>
+        </is>
+      </c>
+      <c r="G67" t="inlineStr">
+        <is>
+          <t>Ronde borstel nylon</t>
+        </is>
+      </c>
+      <c r="H67" t="inlineStr">
+        <is>
+          <t>Messing / Nylon borstelharen</t>
+        </is>
+      </c>
+      <c r="I67" t="inlineStr">
+        <is>
+          <t>Ronde smeerborstel 1 inch voor ketting- en kabeltoepassing inclusief beugel (art. 1414)</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" t="inlineStr">
+        <is>
+          <t>1430</t>
+        </is>
+      </c>
+      <c r="B68" t="inlineStr">
+        <is>
+          <t>Installatiekits</t>
+        </is>
+      </c>
+      <c r="C68" t="inlineStr">
+        <is>
+          <t>Installatiekit 1250RC-1</t>
+        </is>
+      </c>
+      <c r="D68" t="inlineStr">
+        <is>
+          <t>1 smeerpunt</t>
+        </is>
+      </c>
+      <c r="E68" t="inlineStr">
+        <is>
+          <t>Vet</t>
+        </is>
+      </c>
+      <c r="F68" t="inlineStr">
+        <is>
+          <t>Montagebeugel Pulsarlube M</t>
+        </is>
+      </c>
+      <c r="G68" t="inlineStr">
+        <is>
+          <t>Leiding 6 mm + koppeling</t>
+        </is>
+      </c>
+      <c r="H68" t="inlineStr">
+        <is>
+          <t>Verzinkt staal / Polyamide</t>
+        </is>
+      </c>
+      <c r="I68" t="inlineStr">
+        <is>
+          <t>Complete montagekit op afstand voor Pulsarlube M inclusief beugel en koppelingen (art. 1430)</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" t="inlineStr">
+        <is>
+          <t>1415</t>
+        </is>
+      </c>
+      <c r="B69" t="inlineStr">
+        <is>
+          <t>Installatiekits</t>
+        </is>
+      </c>
+      <c r="C69" t="inlineStr">
+        <is>
+          <t>Installatiekit 1 smeerpunt (olie)</t>
+        </is>
+      </c>
+      <c r="D69" t="inlineStr">
+        <is>
+          <t>1 smeerpunt</t>
+        </is>
+      </c>
+      <c r="E69" t="inlineStr">
+        <is>
+          <t>Olie</t>
+        </is>
+      </c>
+      <c r="F69" t="inlineStr">
+        <is>
+          <t>Montagebeugel oliedispenser</t>
+        </is>
+      </c>
+      <c r="G69" t="inlineStr">
+        <is>
+          <t>Leiding 4 mm + koppeling</t>
+        </is>
+      </c>
+      <c r="H69" t="inlineStr">
+        <is>
+          <t>Verzinkt staal / Polyamide</t>
+        </is>
+      </c>
+      <c r="I69" t="inlineStr">
+        <is>
+          <t>Montagekit voor oliesmering 1 smeerpunt (art. 1415)</t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" t="inlineStr">
+        <is>
+          <t>1416</t>
+        </is>
+      </c>
+      <c r="B70" t="inlineStr">
+        <is>
+          <t>Installatiekits</t>
+        </is>
+      </c>
+      <c r="C70" t="inlineStr">
+        <is>
+          <t>Installatiekit 2 smeerpunten (olie)</t>
+        </is>
+      </c>
+      <c r="D70" t="inlineStr">
+        <is>
+          <t>2 smeerpunten</t>
+        </is>
+      </c>
+      <c r="E70" t="inlineStr">
+        <is>
+          <t>Olie</t>
+        </is>
+      </c>
+      <c r="F70" t="inlineStr">
+        <is>
+          <t>Montagebeugel + verdeler 2</t>
+        </is>
+      </c>
+      <c r="G70" t="inlineStr">
+        <is>
+          <t>2x leiding 4 mm + koppelingen</t>
+        </is>
+      </c>
+      <c r="H70" t="inlineStr">
+        <is>
+          <t>Verzinkt staal / Messing</t>
+        </is>
+      </c>
+      <c r="I70" t="inlineStr">
+        <is>
+          <t>Montagekit voor oliesmering 2 smeerpunten (art. 1416)</t>
+        </is>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" t="inlineStr">
+        <is>
+          <t>1417</t>
+        </is>
+      </c>
+      <c r="B71" t="inlineStr">
+        <is>
+          <t>Installatiekits</t>
+        </is>
+      </c>
+      <c r="C71" t="inlineStr">
+        <is>
+          <t>Installatiekit 3 smeerpunten (olie)</t>
+        </is>
+      </c>
+      <c r="D71" t="inlineStr">
+        <is>
+          <t>3 smeerpunten</t>
+        </is>
+      </c>
+      <c r="E71" t="inlineStr">
+        <is>
+          <t>Olie</t>
+        </is>
+      </c>
+      <c r="F71" t="inlineStr">
+        <is>
+          <t>Montagebeugel + verdeler 3</t>
+        </is>
+      </c>
+      <c r="G71" t="inlineStr">
+        <is>
+          <t>3x leiding 4 mm + koppelingen</t>
+        </is>
+      </c>
+      <c r="H71" t="inlineStr">
+        <is>
+          <t>Verzinkt staal / Messing</t>
+        </is>
+      </c>
+      <c r="I71" t="inlineStr">
+        <is>
+          <t>Montagekit voor oliesmering 3 smeerpunten (art. 1417)</t>
+        </is>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" t="inlineStr">
+        <is>
+          <t>1418</t>
+        </is>
+      </c>
+      <c r="B72" t="inlineStr">
+        <is>
+          <t>Installatiekits</t>
+        </is>
+      </c>
+      <c r="C72" t="inlineStr">
+        <is>
+          <t>Installatiekit 4 smeerpunten (olie)</t>
+        </is>
+      </c>
+      <c r="D72" t="inlineStr">
+        <is>
+          <t>4 smeerpunten</t>
+        </is>
+      </c>
+      <c r="E72" t="inlineStr">
+        <is>
+          <t>Olie</t>
+        </is>
+      </c>
+      <c r="F72" t="inlineStr">
+        <is>
+          <t>Montagebeugel + verdeler 4</t>
+        </is>
+      </c>
+      <c r="G72" t="inlineStr">
+        <is>
+          <t>4x leiding 4 mm + koppelingen</t>
+        </is>
+      </c>
+      <c r="H72" t="inlineStr">
+        <is>
+          <t>Verzinkt staal / Messing</t>
+        </is>
+      </c>
+      <c r="I72" t="inlineStr">
+        <is>
+          <t>Montagekit voor oliesmering 4 smeerpunten (art. 1418)</t>
+        </is>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" t="inlineStr">
+        <is>
+          <t>1467</t>
+        </is>
+      </c>
+      <c r="B73" t="inlineStr">
+        <is>
+          <t>Koppelingen &amp; Ventielen</t>
+        </is>
+      </c>
+      <c r="C73" t="inlineStr">
+        <is>
+          <t>Hydraulische terugslagklep 1/8" NPT</t>
+        </is>
+      </c>
+      <c r="D73" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="E73" t="inlineStr">
+        <is>
+          <t>Vet / Olie</t>
+        </is>
+      </c>
+      <c r="F73" t="inlineStr">
+        <is>
+          <t>1/8" NPT M</t>
+        </is>
+      </c>
+      <c r="G73" t="inlineStr">
+        <is>
+          <t>1/8" NPT F</t>
+        </is>
+      </c>
+      <c r="H73" t="inlineStr">
+        <is>
+          <t>Messing vernikkeld</t>
+        </is>
+      </c>
+      <c r="I73" t="inlineStr">
+        <is>
+          <t>Hydraulische terugslagklep voorkomt terugvloeien van smeermiddel (art. 1467)</t>
+        </is>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" t="inlineStr">
+        <is>
+          <t>1453</t>
+        </is>
+      </c>
+      <c r="B74" t="inlineStr">
+        <is>
+          <t>Insteekkoppelingen</t>
+        </is>
+      </c>
+      <c r="C74" t="inlineStr">
+        <is>
+          <t>Push-in koppeling 6 mm x 1/8" NPT M</t>
+        </is>
+      </c>
+      <c r="D74" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="E74" t="inlineStr">
+        <is>
+          <t>Vet / Olie</t>
+        </is>
+      </c>
+      <c r="F74" t="inlineStr">
+        <is>
+          <t>Push-in 6 mm</t>
+        </is>
+      </c>
+      <c r="G74" t="inlineStr">
+        <is>
+          <t>1/8" NPT M</t>
+        </is>
+      </c>
+      <c r="H74" t="inlineStr">
+        <is>
+          <t>Messing vernikkeld</t>
+        </is>
+      </c>
+      <c r="I74" t="inlineStr">
+        <is>
+          <t>Rechte insteekkoppeling voor Pulsarlube verdeelblokken en kits (art. 1453)</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>